<commit_message>
update: service page jsonld format
</commit_message>
<xml_diff>
--- a/docs/page-schemas.xlsx
+++ b/docs/page-schemas.xlsx
@@ -2530,32 +2530,32 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>WebPage; Service; FAQPage; BreadcrumbList</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes — @graph of 3, plus BreadcrumbList emitted separately</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://www.eaststkildadental.com.au/services/&lt;slug&gt;#webpage; https://www.eaststkildadental.com.au/services/&lt;slug&gt;#service; https://www.eaststkildadental.com.au/services/&lt;slug&gt;#faq; https://www.eaststkildadental.com.au/services/&lt;slug&gt;#breadcrumb</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WebPage: url, name (meta title), description (meta description), isPartOf -&gt; #website, about -&gt; #practice, breadcrumb -&gt; #breadcrumb, inLanguage en-AU; Service: serviceType (eyebrow category, e.g. 'General &amp; preventive'), name (meta title without brand), description (meta description), provider -&gt; #practice, areaServed City 'St Kilda East, Victoria, Australia'; FAQPage with 4 Q&amp;A per service from data/services.ts</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes — Home &gt; Services &gt; &lt;Service Name&gt;</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>No JSON-LD written on any of the 20 service pages. Slugs: check-ups, cleans-and-hygiene, childrens-dentistry, mouthguards, tmj-jaw-pain, myofunctional-therapy, fillings, crowns-and-bridges, root-canal, onlays-and-inlays, dentures, extractions-wisdom-teeth, smile-design, veneers, teeth-whitening, invisalign, braces, dental-implants, all-on-4-implants, bone-grafting. Biggest single gap in the audit — each of these is a natural Service node with provider -&gt; #practice.</t>
+          <t>All 20 service pages share one dynamic route (app/services/[slug]/page.tsx), so the markup is identical in shape and differs only in the service's own data from data/services.ts. The @graph mirrors the suburb page pattern: WebPage, Service and FAQPage, each referencing the site-wide #practice and #website entities. No Review or aggregateRating, per AHPRA advertising guidance. Slugs: check-ups, cleans-and-hygiene, childrens-dentistry, mouthguards, tmj-jaw-pain, myofunctional-therapy, fillings, crowns-and-bridges, root-canal, onlays-and-inlays, dentures, extractions-wisdom-teeth, smile-design, veneers, teeth-whitening, invisalign, braces, dental-implants, all-on-4-implants, bone-grafting.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: gaps mentioned in the schema files converted
</commit_message>
<xml_diff>
--- a/docs/page-schemas.xlsx
+++ b/docs/page-schemas.xlsx
@@ -697,22 +697,22 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>MedicalWebPage; BreadcrumbList</t>
+          <t xml:space="preserve">MedicalWebPage; BreadcrumbList</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>No — single node</t>
+          <t xml:space="preserve">No — single node, linked into the site graph by @id reference</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>(none set)</t>
+          <t xml:space="preserve">https://www.eaststkildadental.com.au/learn/&lt;article-slug&gt;#webpage; https://www.eaststkildadental.com.au/learn/&lt;article-slug&gt;#breadcrumb</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>name (article title), author (Person if named, else Organization), publisher (Dentist), inLanguage en-AU, datePublished, dateModified</t>
+          <t xml:space="preserve">name, headline, description (meta description), image, inLanguage en-AU, datePublished, dateModified, isPartOf -&gt; #website, publisher -&gt; #practice, breadcrumb -&gt; #breadcrumb; author -&gt; the reviewing clinician’s Person @id where the byline names one of the four named clinicians, otherwise the #practice node. A name is repeated alongside each @id so the node still reads on its own.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -722,14 +722,14 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Slugs: havent-been-to-the-dentist-in-years, bleeding-gums, how-often-should-you-see-the-dentist, what-to-expect-at-your-first-dental-visit, invisalign-vs-braces-which-is-right-for-you, signs-you-might-be-grinding-your-teeth, dental-implants-vs-bridges-what-you-need-to-know, using-your-superannuation-for-dental-treatment. Gap: no @id, and no isPartOf / publisher @id link back to #website or #practice, so these sit outside the site graph. dateModified is simply copied from datePublished.</t>
+          <t xml:space="preserve">Slugs: havent-been-to-the-dentist-in-years, bleeding-gums, how-often-should-you-see-the-dentist, what-to-expect-at-your-first-dental-visit, invisalign-vs-braces-which-is-right-for-you, signs-you-might-be-grinding-your-teeth, dental-implants-vs-bridges-what-you-need-to-know, using-your-superannuation-for-dental-treatment. dateModified is still copied from datePublished: ArticleData carries no separate updated date.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>/learn/&lt;topic-slug&gt;  (x5)</t>
+          <t xml:space="preserve">/learn/&lt;topic-slug&gt;  (x4)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -744,22 +744,22 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BreadcrumbList only</t>
+          <t xml:space="preserve">CollectionPage; ItemList; BreadcrumbList</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t xml:space="preserve">Yes — @graph of 2, plus BreadcrumbList emitted separately</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>(none set)</t>
+          <t xml:space="preserve">https://www.eaststkildadental.com.au/learn/&lt;topic-slug&gt;#collection; https://www.eaststkildadental.com.au/learn/&lt;topic-slug&gt;#guides; https://www.eaststkildadental.com.au/learn/&lt;topic-slug&gt;#breadcrumb</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Breadcrumb trail only — no CollectionPage or ItemList for the topic's articles</t>
+          <t xml:space="preserve">CollectionPage: url, name, description (the topic intro), isPartOf -&gt; #website, about -&gt; #practice, breadcrumb -&gt; #breadcrumb, mainEntity -&gt; #guides; ItemList: one ListItem per published guide in the topic (position, url, name)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Topics: nervous-patients, prevention, treatments-explained, kids, costs-and-funds. Gap: these list articles on screen but carry no ItemList, unlike the /learn hub.</t>
+          <t xml:space="preserve">Topics with a published guide: nervous-patients, prevention, treatments-explained, costs-and-funds. kids has no published guide, so it has no page and is not in the sitemap. The ItemList is built from guidesByTopic(), the same call that renders the visible grid, so tagging a guide with a topic puts it into the markup with no extra edit.</t>
         </is>
       </c>
     </row>
@@ -1825,32 +1825,32 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t xml:space="preserve">AboutPage; Person x6; Dentist (reference)</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">Yes — @graph of 8</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">https://www.eaststkildadental.com.au/about/our-team#webpage; https://www.eaststkildadental.com.au/about/our-team#&lt;clinician-slug&gt; (x6)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">AboutPage: url, name, description, isPartOf -&gt; #website, about -&gt; #practice, inLanguage en-AU; Person x6: name, jobTitle, description (the visible bio), image, url, worksFor -&gt; #practice; plus a reference to #practice carrying employee -&gt; the 6 Person nodes</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>No JSON-LD written. Team profiles — the Person nodes for these clinicians are declared on the home page graph (@id .../about/our-team#&lt;slug&gt;) but this page emits no JSON-LD of its own.</t>
+          <t xml:space="preserve">This page holds the @id anchors the home page graph references, so it is where the clinicians are described in full. The four named on the home page are the same nodes, restated here with a photo and bio; Dr Marina Bekheet and Beverly Spector are declared here only. jobTitle comes from lib/business.ts wherever that file pins one, which is what keeps Dr Goldman’s markup reading "Dentist" while the visible card says "Dentist &amp; Prosthodontist". The non-clinical practice team is deliberately left out of the markup.</t>
         </is>
       </c>
     </row>
@@ -1919,32 +1919,32 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t xml:space="preserve">CollectionPage; ItemList</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">Yes — @graph of 2</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">https://www.eaststkildadental.com.au/areas-we-serve#collection; https://www.eaststkildadental.com.au/areas-we-serve#suburbs</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">CollectionPage: url, name, description, isPartOf -&gt; #website, about -&gt; #practice, mainEntity -&gt; #suburbs; ItemList: 21 ListItem entries (position, url, name) — St Kilda East (the home page) plus the 20 suburb pages</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>No JSON-LD written. Locations hub linking all 20 suburb pages.</t>
+          <t xml:space="preserve">The ItemList is built from the same areaCards array the visible grid renders, which is itself generated from data/suburbs.ts, so a new suburb page enters the markup with no extra edit.</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>43 page.tsx files, resolving to 71 published URLs (20 suburb + 8 article + 5 topic + 20 service + 18 static)</t>
+          <t xml:space="preserve">43 page.tsx files, resolving to 71 published URLs (20 suburb + 8 article + 4 topic + 20 service + 19 static). Counted from the built sitemap.</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>31 of 71 — home, emergency, /learn, 8 articles, 5 topics (breadcrumb only), 20 suburb pages</t>
+          <t xml:space="preserve">57 of 71 — home, /emergency-dentist, /learn, /areas-we-serve, /about/our-team, 8 articles, 4 topics, 20 suburb pages, 20 service pages</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>40 of 71 — 20 service pages plus 17 static pages, /home redirect, /areas-we-serve, /services hub</t>
+          <t xml:space="preserve">14 of 71 — /about and its two children, /comprehensive-care-visit, /contact, /fees, /nervous-patients, /online-booking, /our-work, /privacy, the /services hub, /terms, /using-your-super, /your-first-visit. The /home redirect and the noindex /take-care-of-you sit outside the 71.</t>
         </is>
       </c>
     </row>
@@ -3035,84 +3035,84 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>GAP — service pages</t>
+          <t xml:space="preserve">RESOLVED — service pages</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>None of the 20 /services/&lt;slug&gt; pages carry a Service node, despite being the site's main commercial pages</t>
+          <t xml:space="preserve">All 20 /services/&lt;slug&gt; pages now carry a WebPage + Service + FAQPage @graph, mirroring the suburb pages.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>GAP — article graph</t>
+          <t xml:space="preserve">RESOLVED — article graph</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>MedicalWebPage on articles has no @id and no isPartOf/publisher @id link, so articles sit outside the site entity graph</t>
+          <t xml:space="preserve">MedicalWebPage now carries an @id, isPartOf -&gt; #website, publisher -&gt; #practice and an author that references the reviewing clinician’s Person @id (or the practice), so articles sit inside the site entity graph. description and image were added at the same time.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>GAP — topic pages</t>
+          <t xml:space="preserve">RESOLVED — topic pages</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>The 5 /learn/&lt;topic&gt; pages list articles but emit no ItemList, unlike /learn</t>
+          <t xml:space="preserve">The 4 populated /learn/&lt;topic&gt; pages now emit CollectionPage + ItemList, built from guidesByTopic() — the same call that renders the visible grid.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>GAP — /areas-we-serve</t>
+          <t xml:space="preserve">RESOLVED — /areas-we-serve</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>The hub linking all 20 suburb pages carries no CollectionPage or ItemList</t>
+          <t xml:space="preserve">The hub now emits CollectionPage + ItemList, built from the same areaCards array the visible grid renders.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>GAP — /about/our-team</t>
+          <t xml:space="preserve">RESOLVED — /about/our-team</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Holds the @id anchors for the 4 Person nodes but emits no markup of its own (nodes are declared on the home page)</t>
+          <t xml:space="preserve">The page now emits AboutPage plus the 6 clinician Person nodes at the @ids it anchors, each with jobTitle, bio, photo and worksFor -&gt; #practice, and an employee list on the #practice reference.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>GAP — sameAs</t>
+          <t xml:space="preserve">OPEN — sameAs</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>lib/business.ts has TODOs for Facebook, Instagram and HealthEngine URLs — the sameAs array is incomplete</t>
+          <t xml:space="preserve">lib/business.ts still has TODOs for the Facebook, Instagram and HealthEngine URLs — sameAs holds only the Google Business Profile link. Needs the URLs from the practice; placeholders are deliberately not shipped.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>GAP — geo</t>
+          <t xml:space="preserve">OPEN — geo</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>lib/business.ts flags latitude/longitude as taken from an SEO recommendation, not verified against the Google Business Profile</t>
+          <t xml:space="preserve">lib/business.ts still flags latitude/longitude as taken from an SEO recommendation, not verified against the Google Business Profile. Needs someone with access to the live GBP listing to confirm or correct them.</t>
         </is>
       </c>
     </row>

</xml_diff>